<commit_message>
Update Base 10 Ha production with real field data
Field survey revealed actual production from existing 1,500 plants:
- 2028: 2,000 poles (was 1,000)
- 2029: 3,500 poles (steady state from existing plants)
- 2030: 3,500 poles
- 2031: 3,500 poles (transition year - new plants just mature)
- 2032: 10,500 poles (new 3,500 plants yr6)
- 2033+: 14,000 poles (all 5,000 plants fully mature)

Plant density update:
- Existing 1,500 plants on 10 ha (~150/ha actual)
- Plant 3,500 new seedlings in 2026 to densify to 500/ha target
- New plants reach maturity in 2031 (5 years from planting)
- Total density achieved: 5,000 plants = 500/ha by 2033

Base 10 ha revenue progression:
- 2028-2031: 680K-1.19M MXN (from existing plants)
- 2032: 3.57M MXN (densification kicks in)
- 2033+: 4.76M MXN (full maturity)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pacifico_Bambu_Financial_Model_v2.xlsx
+++ b/Pacifico_Bambu_Financial_Model_v2.xlsx
@@ -1971,22 +1971,22 @@
       </c>
       <c r="C133" s="23" t="inlineStr">
         <is>
-          <t>Survey: 1,500 healthy plants on 10 ha</t>
+          <t>Existing plants on 10 ha (~150/ha)</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="23" t="inlineStr">
         <is>
-          <t>Target plants per ha</t>
+          <t>NEW seedlings to plant 2026 (densify)</t>
         </is>
       </c>
       <c r="B134" s="23" t="n">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="C134" s="23" t="inlineStr">
         <is>
-          <t>After densification</t>
+          <t>1500 existing + 3500 new = 5000 (500/ha)</t>
         </is>
       </c>
     </row>
@@ -2027,11 +2027,11 @@
         </is>
       </c>
       <c r="B137" s="23" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="C137" s="23" t="inlineStr">
         <is>
-          <t>1,000 plants reach maturity (yr5)</t>
+          <t>Existing 1500 plants in yr5</t>
         </is>
       </c>
     </row>
@@ -2042,11 +2042,11 @@
         </is>
       </c>
       <c r="B138" s="23" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="C138" s="23" t="inlineStr">
         <is>
-          <t>1,000 yr6 (2/plant) + 500 yr5 (1/plant)</t>
+          <t>Steady state from 1500 existing plants</t>
         </is>
       </c>
     </row>
@@ -2057,11 +2057,11 @@
         </is>
       </c>
       <c r="B139" s="23" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="C139" s="23" t="inlineStr">
         <is>
-          <t>1,000 yr7+ (4/plant) + 500 yr6 (2/plant)</t>
+          <t>Steady state from existing</t>
         </is>
       </c>
     </row>
@@ -2072,11 +2072,11 @@
         </is>
       </c>
       <c r="B140" s="23" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
       <c r="C140" s="23" t="inlineStr">
         <is>
-          <t>Steady state: 1,500 plants × 4 poles</t>
+          <t>After 2031: ALL 5000 plants mature (1500+3500)</t>
         </is>
       </c>
     </row>
@@ -2763,9 +2763,8 @@
       <c r="A7" s="11" t="n">
         <v>2031</v>
       </c>
-      <c r="B7" s="12">
-        <f>Assumptions!$B$140</f>
-        <v/>
+      <c r="B7" s="12" t="n">
+        <v>3500</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>0</v>
@@ -2808,9 +2807,8 @@
       <c r="A8" s="11" t="n">
         <v>2032</v>
       </c>
-      <c r="B8" s="12">
-        <f>Assumptions!$B$140</f>
-        <v/>
+      <c r="B8" s="12" t="n">
+        <v>10500</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>0</v>
@@ -3763,7 +3761,7 @@
         <v>2026</v>
       </c>
       <c r="B2" s="9">
-        <f>3000*Assumptions!$B$18</f>
+        <f>Assumptions!$B$134*Assumptions!$B$18</f>
         <v/>
       </c>
       <c r="C2" s="9">

</xml_diff>

<commit_message>
Set conservative base yield 1,400 poles/ha (was 2,000)
Rationale: Be defensible to investors. Published research shows Guadua
bamboo yields range widely (800-3,000 poles/ha). We use 1,400 as base
case — comfortably within realistic range, not overly optimistic.

Changes:
- Excel Assumptions B4-B6: yr5=350, yr6=700, yr7+=1,400 (was 500/1000/2000)
- Base 10 ha steady state remains 14,000 poles (10 × 1,400) — consistent
- Full 110 ha maturity: 154,000 poles/year (was 220,000)
- Revenue 2038: 52M MXN (was 73M) — more defensible

Sensitivity scenarios (PPTX + HTML):
- Conservative: 1,000/ha — downside protection
- Base Case ⭐: 1,400/ha — OUR PROJECTION
- Optimistic: 2,000-3,000/ha — possible upside

Prominently noted on Financial Projections and Sensitivity slides.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pacifico_Bambu_Financial_Model_v2.xlsx
+++ b/Pacifico_Bambu_Financial_Model_v2.xlsx
@@ -595,7 +595,12 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>500</v>
+        <v>350</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Year 5 first production (25% of mature)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -605,17 +610,27 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1000</v>
+        <v>700</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Year 6 scaling (50% of mature)</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Yield yr7+ (poles/ha)</t>
+          <t>Yield yr7+ (BASE: 1,400/ha)</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>2000</v>
+        <v>1400</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>⚠ CONSERVATIVE BASE (range: 1,000-2,000-3,000)</t>
+        </is>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Align deck + financial model with refined export and carbon strategy
Deck (docs/index.html):
- Slide 5: clarify carbon credits as via partner (zero cost)
- Slide 15: replace generic "Verra registration" with carbon partnership
  milestone (revenue share, partner does technical work) + optional
  in-house transition post-2033

Financial model (Excel):
- Bridge round: 2M -> 4M MXN (matches deck Round 1)
- Seed round: 3M -> 5M MXN (matches deck Round 2)
- Dividend start year: 2030 -> 2033 (matches cumulative break-even)
- Carbon verification cost (B122): 50K/year -> 0 (partner covers cost)
- Carbon revenue stream activated 2028+ via 50% partner share formula

Scripts:
- Add update_fx_rate.py for daily MXN/USD rate refresh from
  open.er-api.com with Yahoo Finance fallback. Backs up Excel before
  writing. Run with --dry-run to preview.

Verified: 662 formulas intact, zero errors after changes.
</commit_message>
<xml_diff>
--- a/Pacifico_Bambu_Financial_Model_v2.xlsx
+++ b/Pacifico_Bambu_Financial_Model_v2.xlsx
@@ -662,6 +662,11 @@
       <c r="B7" s="5" t="n">
         <v>21</v>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Net to Pacifico after partner revenue share (~50%)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -670,7 +675,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>17</v>
+        <v>17.4103</v>
       </c>
     </row>
     <row r="9">
@@ -680,7 +685,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>2000000</v>
+        <v>4000000</v>
       </c>
     </row>
     <row r="10">
@@ -690,7 +695,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>3000000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="11">
@@ -790,7 +795,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>2030</v>
+        <v>2033</v>
       </c>
     </row>
     <row r="21">
@@ -1879,11 +1884,11 @@
         </is>
       </c>
       <c r="B122" s="23" t="n">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="C122" s="23" t="inlineStr">
         <is>
-          <t>Verra process</t>
+          <t>Partner pays — set &gt;0 only if going in-house post-2033</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1903,7 @@
       </c>
       <c r="C123" s="23" t="inlineStr">
         <is>
-          <t>After plantation matures</t>
+          <t>Optional in-house start (decision based on economics)</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3200,7 @@
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>Carbon Credits (0, external)</t>
+          <t>Carbon Credits (50% partner share)</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
@@ -3236,8 +3241,10 @@
         <f>B2*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D2" s="9" t="n">
-        <v>0</v>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E2" s="9" t="n">
         <v>0</v>
@@ -3271,8 +3278,10 @@
         <f>B3*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D3" s="9" t="n">
-        <v>0</v>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E3" s="9" t="n">
         <v>0</v>
@@ -3306,8 +3315,9 @@
         <f>B4*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D4" s="9" t="n">
-        <v>0</v>
+      <c r="D4" s="9">
+        <f>Assumptions!$C$35*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E4" s="9" t="n">
         <v>0</v>
@@ -3341,8 +3351,9 @@
         <f>B5*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D5" s="9" t="n">
-        <v>0</v>
+      <c r="D5" s="9">
+        <f>Assumptions!$C$36*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E5" s="9" t="n">
         <v>0</v>
@@ -3376,8 +3387,9 @@
         <f>B6*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>0</v>
+      <c r="D6" s="9">
+        <f>Assumptions!$C$37*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E6" s="9">
         <f>(A6-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3412,8 +3424,9 @@
         <f>B7*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>0</v>
+      <c r="D7" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E7" s="9">
         <f>(A7-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3448,8 +3461,9 @@
         <f>B8*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>0</v>
+      <c r="D8" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E8" s="9">
         <f>(A8-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3484,8 +3498,9 @@
         <f>B9*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>0</v>
+      <c r="D9" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E9" s="9">
         <f>(A9-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3520,8 +3535,9 @@
         <f>B10*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>0</v>
+      <c r="D10" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E10" s="9">
         <f>(A10-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3556,8 +3572,9 @@
         <f>B11*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>0</v>
+      <c r="D11" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E11" s="9">
         <f>(A11-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3592,8 +3609,9 @@
         <f>B12*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>0</v>
+      <c r="D12" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E12" s="9">
         <f>(A12-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3628,8 +3646,9 @@
         <f>B13*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D13" s="9" t="n">
-        <v>0</v>
+      <c r="D13" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E13" s="9">
         <f>(A13-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>
@@ -3664,8 +3683,9 @@
         <f>B14*Assumptions!$B$2</f>
         <v/>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>0</v>
+      <c r="D14" s="9">
+        <f>Assumptions!$C$38*Assumptions!$B$7*0.5*Assumptions!$B$8</f>
+        <v/>
       </c>
       <c r="E14" s="9">
         <f>(A14-Assumptions!$B$151+1)*Assumptions!$B$150*Assumptions!$B$17</f>

</xml_diff>

<commit_message>
Fix Rick role + add export prep / logistics expense lines
Deck (slide 10):
- Replace "Series A funds Export Director + QC Manager" with
  "Operating cash flow (2034+) funds Export Director + QC Manager
  as ICC-ES 2037 approaches" — Rick is angel only, no Series A in plan.

Excel financial model:
- Add Assumptions rows 175-186 with new Export Prep & Logistics params:
  - ASTM bench tests: 200K MXN one-time (2028, from Round 2 earmark)
  - FSC Chain of Custody: 100K initial (2031) + 60K/yr ongoing
  - Pack 1 setup: 140K MXN one-time (2036)
  - Pack 1 per-container logistics: 25K MXN x 4 containers/yr (2037+)
- Update Expenses!J (Consulting & Tech) formula to include all new items.
- Pack 2 ICC-ES 2.5M Capex (2037) already existed — left intact.

Verified: 664 formulas, zero errors.
</commit_message>
<xml_diff>
--- a/Pacifico_Bambu_Financial_Model_v2.xlsx
+++ b/Pacifico_Bambu_Financial_Model_v2.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C171"/>
+  <dimension ref="A1:C186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -808,6 +808,7 @@
         <v>0.1</v>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
@@ -865,6 +866,7 @@
         <v>0.2</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -1247,6 +1249,7 @@
       <c r="A66" s="18" t="n"/>
       <c r="B66" s="3" t="n"/>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="18" t="n"/>
       <c r="B68" s="9" t="n"/>
@@ -1255,6 +1258,8 @@
       <c r="A69" s="18" t="n"/>
       <c r="B69" s="9" t="n"/>
     </row>
+    <row r="70"/>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="21" t="inlineStr">
         <is>
@@ -1356,6 +1361,7 @@
         </is>
       </c>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" s="21" t="inlineStr">
         <is>
@@ -1410,6 +1416,7 @@
         </is>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="21" t="inlineStr">
         <is>
@@ -1480,6 +1487,7 @@
         </is>
       </c>
     </row>
+    <row r="90"/>
     <row r="91">
       <c r="A91" s="21" t="inlineStr">
         <is>
@@ -1595,6 +1603,7 @@
         </is>
       </c>
     </row>
+    <row r="99"/>
     <row r="100">
       <c r="A100" s="21" t="inlineStr">
         <is>
@@ -1664,6 +1673,7 @@
         </is>
       </c>
     </row>
+    <row r="105"/>
     <row r="106">
       <c r="A106" s="21" t="inlineStr">
         <is>
@@ -1793,6 +1803,7 @@
         </is>
       </c>
     </row>
+    <row r="115"/>
     <row r="116">
       <c r="A116" s="21" t="inlineStr">
         <is>
@@ -1907,6 +1918,7 @@
         </is>
       </c>
     </row>
+    <row r="124"/>
     <row r="125">
       <c r="A125" s="21" t="inlineStr">
         <is>
@@ -1976,6 +1988,7 @@
         </is>
       </c>
     </row>
+    <row r="130"/>
     <row r="131">
       <c r="A131" s="21" t="inlineStr">
         <is>
@@ -2120,6 +2133,7 @@
         </is>
       </c>
     </row>
+    <row r="141"/>
     <row r="142">
       <c r="A142" s="21" t="inlineStr">
         <is>
@@ -2189,6 +2203,7 @@
         </is>
       </c>
     </row>
+    <row r="147"/>
     <row r="148">
       <c r="A148" s="21" t="inlineStr">
         <is>
@@ -2434,6 +2449,7 @@
         </is>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
@@ -2466,6 +2482,183 @@
       </c>
       <c r="B171" t="n">
         <v>2033</v>
+      </c>
+    </row>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>EXPORT PREP &amp; LOGISTICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>ASTM bench tests cost (one-time)</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>~$11K — Phase 1 of Pack 2, paid 2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>ASTM start year</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>From Round 2 earmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>FSC Chain of Custody initial</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>~$6K initial cert — paid 2031</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>FSC annual maintenance</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>~$3.5K/year ongoing audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>FSC start year</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>2031</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>When pre-export prep deepens</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Pack 1 setup (one-time)</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>140000</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>SEMARNAT + Padron + APHIS + setup ~$8K</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Pack 1 setup year</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>2036</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>12 months before first export</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Pack 1 per-container cost</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>~$1.5K/container — phyto + heat + broker + freight share</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Containers per year (assumed)</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>4</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Conservative 2037; scales after</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Pack 1 logistics start year</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>2037</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>First export year</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3846,8 +4039,9 @@
         <f>Production!L2*Assumptions!$B$129</f>
         <v/>
       </c>
-      <c r="J2" s="12" t="n">
-        <v>0</v>
+      <c r="J2" s="12">
+        <f>IF(A2&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A2&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A2=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A2=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A2&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A2=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A2&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
+        <v/>
       </c>
       <c r="K2" s="10">
         <f>SUM(B2:J2)+L2+O2</f>
@@ -3902,8 +4096,9 @@
         <f>Production!L3*Assumptions!$B$129</f>
         <v/>
       </c>
-      <c r="J3" s="12" t="n">
-        <v>0</v>
+      <c r="J3" s="12">
+        <f>IF(A3&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A3&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A3=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A3=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A3&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A3=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A3&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
+        <v/>
       </c>
       <c r="K3" s="10">
         <f>SUM(B3:J3)+L3+O3</f>
@@ -3960,7 +4155,7 @@
         <v/>
       </c>
       <c r="J4" s="12">
-        <f>IF(A4&gt;=Assumptions!$B$121,Assumptions!$B$120,0)</f>
+        <f>IF(A4&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A4&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A4=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A4=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A4&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A4=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A4&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K4" s="10">
@@ -4019,7 +4214,7 @@
         <v/>
       </c>
       <c r="J5" s="12">
-        <f>IF(A5&gt;=Assumptions!$B$121,Assumptions!$B$120,0)</f>
+        <f>IF(A5&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A5&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A5=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A5=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A5&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A5=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A5&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K5" s="10">
@@ -4079,7 +4274,7 @@
         <v/>
       </c>
       <c r="J6" s="12">
-        <f>IF(A6&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A6&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A6&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A6&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A6=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A6=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A6&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A6=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A6&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K6" s="10">
@@ -4139,7 +4334,7 @@
         <v/>
       </c>
       <c r="J7" s="12">
-        <f>IF(A7&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A7&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A7&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A7&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A7=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A7=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A7&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A7=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A7&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K7" s="10">
@@ -4198,7 +4393,7 @@
         <v/>
       </c>
       <c r="J8" s="12">
-        <f>IF(A8&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A8&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A8&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A8&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A8=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A8=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A8&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A8=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A8&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K8" s="10">
@@ -4256,7 +4451,7 @@
         <v/>
       </c>
       <c r="J9" s="12">
-        <f>IF(A9&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A9&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A9&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A9&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A9=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A9=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A9&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A9=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A9&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K9" s="10">
@@ -4314,7 +4509,7 @@
         <v/>
       </c>
       <c r="J10" s="12">
-        <f>IF(A10&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A10&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A10&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A10&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A10=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A10=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A10&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A10=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A10&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K10" s="10">
@@ -4372,7 +4567,7 @@
         <v/>
       </c>
       <c r="J11" s="12">
-        <f>IF(A11&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A11&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A11&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A11&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A11=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A11=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A11&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A11=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A11&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K11" s="10">
@@ -4431,7 +4626,7 @@
         <v/>
       </c>
       <c r="J12" s="12">
-        <f>IF(A12&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A12&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A12&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A12&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A12=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A12=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A12&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A12=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A12&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K12" s="10">
@@ -4490,7 +4685,7 @@
         <v/>
       </c>
       <c r="J13" s="12">
-        <f>IF(A13&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A13&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A13&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A13&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A13=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A13=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A13&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A13=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A13&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K13" s="10">
@@ -4549,7 +4744,7 @@
         <v/>
       </c>
       <c r="J14" s="12">
-        <f>IF(A14&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A14&gt;=Assumptions!$B$123,Assumptions!$B$122,0)</f>
+        <f>IF(A14&gt;=Assumptions!$B$121,Assumptions!$B$120,0)+IF(A14&gt;=Assumptions!$B$123,Assumptions!$B$122,0)+IF(A14=Assumptions!$B$178,Assumptions!$B$177,0)+IF(A14=Assumptions!$B$181,Assumptions!$B$179,0)+IF(A14&gt;Assumptions!$B$181,Assumptions!$B$180,0)+IF(A14=Assumptions!$B$183,Assumptions!$B$182,0)+IF(A14&gt;=Assumptions!$B$186,Assumptions!$B$184*Assumptions!$B$185,0)</f>
         <v/>
       </c>
       <c r="K14" s="10">

</xml_diff>